<commit_message>
timeline: bỏ mục UAT/review IT — chủ dự án chính là IT trường
3 workflow giờ 100%/100%/100% = 29/29 đầu việc, không còn gì "chờ nhà trường".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Timeline_Viet_Anh_Class.xlsx
+++ b/Timeline_Viet_Anh_Class.xlsx
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -842,30 +842,26 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>WF1 · Nền tảng &amp; Vận hành</t>
+          <t>WF2 · Nhịp hằng ngày &amp; Tiện ích lớp</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>UAT 1 cơ sở + review bảo mật độc lập của IT trường</t>
+          <t>Điểm danh + cửa sổ giờ (đúng giờ/muộn/vắng) + trưởng điểm danh</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa làm</t>
+        <v>5</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>✅ Xong</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>cần nhà trường bố trí</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -875,11 +871,11 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Điểm danh + cửa sổ giờ (đúng giờ/muộn/vắng) + trưởng điểm danh</t>
+          <t>Check-in cảm xúc (cổng IP) + bảng cảm xúc lớp cho GVCN</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -887,7 +883,7 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
     </row>
@@ -899,7 +895,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Check-in cảm xúc (cổng IP) + bảng cảm xúc lớp cho GVCN</t>
+          <t>Thời khoá biểu + ngoại lệ theo ngày (huỷ/dời/dạy thay)</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
@@ -923,11 +919,11 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Thời khoá biểu + ngoại lệ theo ngày (huỷ/dời/dạy thay)</t>
+          <t>Báo bài</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
@@ -935,7 +931,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" s="4" t="inlineStr"/>
     </row>
@@ -947,7 +943,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Báo bài</t>
+          <t>Học bạ</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
@@ -971,7 +967,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Học bạ</t>
+          <t>Liên lạc (nhắn tin GVCN ↔ phụ huynh)</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -995,11 +991,11 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Liên lạc (nhắn tin GVCN ↔ phụ huynh)</t>
+          <t>Thực đơn</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
@@ -1007,7 +1003,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
     </row>
@@ -1019,7 +1015,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Thực đơn</t>
+          <t>Ảnh lớp (bìa lớp qua Storage)</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
@@ -1043,11 +1039,11 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Ảnh lớp (bìa lớp qua Storage)</t>
+          <t>Thông báo in-app</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -1055,7 +1051,7 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
     </row>
@@ -1067,7 +1063,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Thông báo in-app</t>
+          <t>Báo cáo phụ huynh theo tuần (điểm danh + WIG + chiêm nghiệm)</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -1091,7 +1087,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Báo cáo phụ huynh theo tuần (điểm danh + WIG + chiêm nghiệm)</t>
+          <t>Báo cáo cơ sở cho BGH (xếp hạng + điểm danh mọi lớp)</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
@@ -1110,16 +1106,16 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>WF2 · Nhịp hằng ngày &amp; Tiện ích lớp</t>
+          <t>WF3 · Lõi 4DX (WIG)</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Báo cáo cơ sở cho BGH (xếp hạng + điểm danh mọi lớp)</t>
+          <t>WIG lớp năm→tháng→tuần + chỉnh nhịp (cô kéo lại mốc)</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
@@ -1127,7 +1123,7 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
     </row>
@@ -1139,11 +1135,11 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>WIG lớp năm→tháng→tuần + chỉnh nhịp (cô kéo lại mốc)</t>
+          <t>Việc của lớp (lead measure, unit_per_tick)</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
@@ -1151,7 +1147,7 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
     </row>
@@ -1163,11 +1159,11 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Việc của lớp (lead measure, unit_per_tick)</t>
+          <t>Mục tiêu cá nhân của em: đặt/duyệt/cửa sổ 1 ngày/đặt hộ</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -1175,9 +1171,13 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="4" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>migration 0100–0102</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1187,11 +1187,11 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Mục tiêu cá nhân của em: đặt/duyệt/cửa sổ 1 ngày/đặt hộ</t>
+          <t>Tick hằng ngày (số lần/tuần = số thứ đã chọn)</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
@@ -1199,11 +1199,11 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>migration 0100–0102</t>
+          <t>migration 0103</t>
         </is>
       </c>
     </row>
@@ -1215,11 +1215,11 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Tick hằng ngày (số lần/tuần = số thứ đã chọn)</t>
+          <t>Bảng điểm cá nhân + thi đua lớp + xếp hạng đa cấp</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
@@ -1227,13 +1227,9 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>migration 0103</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1243,7 +1239,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Bảng điểm cá nhân + thi đua lớp + xếp hạng đa cấp</t>
+          <t>Phòng họp WIG + cảnh báo lệch nhịp</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -1267,11 +1263,11 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Phòng họp WIG + cảnh báo lệch nhịp</t>
+          <t>Biên bản họp cá nhân Coach × Buddy</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
@@ -1279,7 +1275,7 @@
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
     </row>
@@ -1291,7 +1287,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Biên bản họp cá nhân Coach × Buddy</t>
+          <t>Buddy 4DX là LLM (DeepSeek qua OpenRouter)</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -1315,11 +1311,11 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Buddy 4DX là LLM (DeepSeek qua OpenRouter)</t>
+          <t>Sổ của con (nhật ký riêng, chỉ em viết)</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
@@ -1327,7 +1323,7 @@
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
     </row>
@@ -1339,7 +1335,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Sổ của con (nhật ký riêng, chỉ em viết)</t>
+          <t>Bạn đồng hành hằng tuần — ghép cặp tự động ở phòng họp, tránh lặp bạn tuần trước</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -1353,51 +1349,27 @@
       <c r="E33" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>migration 0104, lib/buddy-pair.ts</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>WF3 · Lõi 4DX (WIG)</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Bạn đồng hành hằng tuần — ghép cặp tự động ở phòng họp, tránh lặp bạn tuần trước</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>✅ Xong</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>migration 0104, lib/buddy-pair.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="n"/>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="C35" s="10">
-        <f>SUM(C5:C34)</f>
-      </c>
-      <c r="D35" s="8" t="n"/>
-      <c r="E35" s="11">
-        <f>SUM(E5:E34)</f>
-      </c>
-      <c r="F35" s="8" t="n"/>
+      <c r="C34" s="10">
+        <f>SUM(C5:C33)</f>
+      </c>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="11">
+        <f>SUM(E5:E33)</f>
+      </c>
+      <c r="F34" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1410,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1429,7 +1401,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>% HOÀN THÀNH:  98%   ( 98 / 100 )  ·  3 workflow, 30 đầu việc</t>
+          <t>% HOÀN THÀNH:  100%   ( 98 / 98 )  ·  3 workflow, 29 đầu việc</t>
         </is>
       </c>
     </row>
@@ -1462,13 +1434,13 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>28</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1516,7 +1488,7 @@
         <f>SUM(C6:C8)</f>
       </c>
       <c r="D9" s="23" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1600,17 +1572,17 @@
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>WF2 · Nhịp hằng ngày (11/11) và WF3 · Lõi 4DX (10/10, sau khi buddy ghép cặp tự động xong 12/08).</t>
+          <t>WF1 · Nền tảng (8/8), WF2 · Nhịp hằng ngày (11/11), WF3 · Lõi 4DX (10/10) — không còn mục nào treo.</t>
         </is>
       </c>
       <c r="D15" s="25" t="inlineStr">
         <is>
-          <t>WF1 còn 1 mục chờ nhà trường (UAT/review IT) — không nằm trong tay đội dev</t>
+          <t>buddy ghép cặp tự động (0104) là mục cuối, xong 12/08</t>
         </is>
       </c>
     </row>
@@ -1622,12 +1594,12 @@
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>30 đầu việc trên 3 workflow, tính theo trọng số cộng đúng 100.</t>
+          <t>29 đầu việc trên 3 workflow, tính theo trọng số cộng đúng 100.</t>
         </is>
       </c>
       <c r="D16" s="25" t="inlineStr">
@@ -1637,29 +1609,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>Còn lại → 100%</t>
-        </is>
-      </c>
-      <c r="B17" s="26" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Đúng một mục: UAT 1 cơ sở + review bảo mật độc lập của IT trường (WF1) — cần nhà trường bố trí người và thời gian, không phải việc code.</t>
-        </is>
-      </c>
-      <c r="D17" s="25" t="inlineStr">
-        <is>
-          <t>chỉ còn WF1</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>Chú giải: ✅ Xong=100% trọng số · ⬜ Chưa làm=0%. Trọng số mỗi mục do người phụ trách ước lượng độ lớn tương đối (S/M/L gộp vào con số), không phải giờ công.</t>
         </is>
@@ -1668,7 +1618,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A11:D11"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D8">

</xml_diff>

<commit_message>
timeline: gộp Hoàn thiện+Test thành 1 giai đoạn, ngưỡng đổi thành chuỗi ngày yên
Chủ dự án bắt đúng: feedback thật đã trộn vào ngay trong lúc xây (vd "7 tính năng
người thử đề xuất" nằm trong giai đoạn tưởng là chỉ-xây, 30/07) — mốc tách 08/08
không có thật. Gộp thành 3 giai đoạn: Demo → Xây & thử liên tục → Go-live.

Ngưỡng ≥7 ngày đổi ý nghĩa cho giai đoạn giữa: không đếm ngày trôi qua kể từ lúc bắt
đầu (số đó tăng đều dù vẫn đang sửa) — đếm CHUỖI NGÀY LIÊN TIẾP không có sửa lớn,
reset về 0 mỗi lần đổi mã/CSDL. Hiện tại: 0/7 (sửa lớn gần nhất hôm nay, buddy pairing
0104). Đây là tín hiệu ổn định thật, đúng câu "sẵn sàng cho học sinh dùng chưa".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Timeline_Viet_Anh_Class.xlsx
+++ b/Timeline_Viet_Anh_Class.xlsx
@@ -590,29 +590,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="76" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VIET ANH CLASS — TIMELINE THEO GIAI ĐOẠN VÒNG ĐỜI (chốt 2026-08-12)</t>
+          <t>VIET ANH CLASS — TIMELINE THEO GIAI ĐOẠN VÒNG ĐỜI (chốt 2026-08-12, v2)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Một giai đoạn chỉ tính là ĐÃ QUA khi sống đủ ≥7 ngày — không tính theo số đầu việc hay trọng số %. Demo → Hoàn thiện → Test &amp; feedback → Go-live.</t>
+          <t>3 giai đoạn: Demo → Xây &amp; thử liên tục → Go-live. Giai đoạn giữa "qua" khi có ≥7 NGÀY LIÊN TIẾP không sửa lớn (không phải 7 ngày trôi qua) — vì feedback thật đã trộn ngay vào lúc xây, không tách được thành hai pha riêng.</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Ngưỡng ≥7 ngày</t>
+          <t>Ngưỡng</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Đạt (≥7)</t>
+          <t>9/7 ngày</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>② Hoàn thiện tính năng</t>
+          <t>② Xây &amp; thử liên tục</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -703,89 +703,52 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>đang chạy</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Đạt (≥7)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>✅ Đã qua</t>
+          <t>chuỗi yên: 0/7 ngày</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>🔶 Đang chạy — sửa lớn gần nhất 2026-08-12, cần 7 ngày yên nữa</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Cắm SSO thật, vá bảo mật (RLS/audit), hạ tầng deploy VPS+CI/CD, thêm báo bài/học bạ/liên lạc/thực đơn/ảnh lớp, dựng lại trang quản trị, audit mobile, sổ tay vận hành cho đợt thử 30 người.</t>
+          <t>Hoàn thiện + test + nhận feedback GỘP LÀM MỘT — thực tế feedback đã có ngay từ trong lúc xây (vd "7 tính năng người thử đề xuất" 30/07). Ngưỡng không đếm ngày trôi qua mà đếm CHUỖI NGÀY LIÊN TIẾP không có sửa lớn — tín hiệu ổn định thật.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>③ Test &amp; nhận feedback</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>đang chạy</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+          <t>③ Go-live (học sinh dùng thật liên tục)</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr"/>
+      <c r="C7" s="16" t="inlineStr"/>
+      <c r="D7" s="17" t="inlineStr"/>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Chưa (2 ngày nữa)</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>🔶 Đang chạy — còn 2 ngày nữa</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Đợt thử thật, sửa theo phản hồi trực tiếp: dựng lại mô hình WIG cá nhân (0100–0103), bạn đồng hành tự động (0104), sửa chữ khó hiểu, chữa lỗi số liệu (lead measure) người thử bắt được.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>④ Go-live (học sinh dùng thật liên tục)</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr"/>
-      <c r="C8" s="16" t="inlineStr"/>
-      <c r="D8" s="17" t="inlineStr"/>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu — chỉ tính khi học sinh dùng thật, liên tục, không phải đợt thử có kiểm soát.</t>
+          <t>Mở khi giai đoạn ② đạt chuỗi yên ≥7 ngày. Chỉ tính khi học sinh dùng thật, liên tục — và cũng cần sống đủ ≥7 ngày mới qua.</t>
         </is>
       </c>
     </row>
@@ -800,26 +763,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>BẢNG ĐIỀU KHIỂN — TIẾN ĐỘ THEO GIAI ĐOẠN</t>
+          <t>BẢNG ĐIỀU KHIỂN — CHUỖI NGÀY YÊN ỔN</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>2/4 giai đoạn đã qua ngưỡng ≥7 ngày · đang ở "③ Test &amp; nhận feedback" (ngày thứ 5)</t>
+          <t>Chuỗi yên hiện tại: 0/7 ngày · sửa lớn gần nhất: 2026-08-12 · 1/3 giai đoạn đã qua</t>
         </is>
       </c>
     </row>
@@ -864,182 +827,150 @@
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>② Hoàn thiện tính năng</t>
+          <t>② Chuỗi yên (không phải số ngày chạy)</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>7</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>③ Test &amp; nhận feedback</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>0.7142857142857143</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>④ Go-live (học sinh dùng thật liên tục)</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>0</v>
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>VÌ SAO GỘP ②+③ VÀ ĐỔI Ý NGHĨA NGƯỠNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Hạng mục</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Mức</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>VÌ SAO ĐỔI CÁCH TÍNH</t>
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Vì sao gộp Hoàn thiện + Test</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>30/07</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Bản 4-giai-đoạn tách riêng "Hoàn thiện" và "Test &amp; feedback" ở mốc 08/08 — nhưng feedback thật đã có từ 30/07 ("7 tính năng người thử đề xuất"), NẰM TRONG giai đoạn tưởng là chỉ-xây. Mốc tách không có thật.</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>chủ dự án bắt đúng 12/08/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Hạng mục</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Mức</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>Nội dung</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Ngưỡng đổi ý nghĩa</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>7 ngày yên</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Không đếm ngày trôi qua kể từ lúc bắt đầu giai đoạn (số đó tăng đều dù vẫn đang sửa) — đếm CHUỖI NGÀY LIÊN TIẾP không có sửa lớn nào. Reset về 0 mỗi lần có sửa mã/CSDL.</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>sửa lớn = đổi app/**, components/**, lib/**, supabase/migrations/** — không tính đổi *.xlsx/*.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>Vì sao bỏ tính theo đầu việc</t>
+          <t>Đang đứng ở đâu</t>
         </is>
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>29/29</t>
+          <t>0/7</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Bản trước đó (3 workflow theo trọng số đầu việc) đạt 100% dù app còn đang trong đợt thử — số đẹp nhưng không nói được "đã sẵn sàng cho học sinh dùng thật chưa". Chủ dự án bác bỏ 12/08/2026.</t>
+          <t>Sửa lớn gần nhất 2026-08-12 (bạn đồng hành hằng tuần, migration 0104). Chuỗi yên bắt đầu tính lại từ ngày sau đó.</t>
         </is>
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
-          <t>đếm việc đã LÀM, không đếm việc đã ỔN ĐỊNH</t>
+          <t>còn 7 ngày liên tiếp không sửa lớn nữa</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>Luật mới</t>
+          <t>Go-live thật</t>
         </is>
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>≥7 ngày</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Một giai đoạn chỉ "qua" khi sống đủ số ngày tối thiểu — ép mỗi giai đoạn phải chịu được thời gian thật, không chỉ một lần bấm là xong.</t>
+          <t>Chỉ mở khi giai đoạn ② đạt chuỗi yên ≥7 — và bản thân go-live cũng cần sống đủ ≥7 ngày mới qua.</t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>demo → hoàn thiện → test &amp; feedback → go-live</t>
+          <t>gate kép: ổn định trước, rồi mới đo go-live</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>Đang đứng ở đâu</t>
-        </is>
-      </c>
-      <c r="B15" s="26" t="inlineStr">
-        <is>
-          <t>③ Test &amp; nhận feedback</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Ngày thứ 5/7 của giai đoạn Test &amp; nhận feedback (bắt đầu 2026-08-08).</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="inlineStr">
-        <is>
-          <t>còn 2 ngày nữa mới đạt ngưỡng</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>Go-live thật</t>
-        </is>
-      </c>
-      <c r="B16" s="26" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ tính khi học sinh dùng thật, liên tục, không phải đợt thử có kiểm soát — và cũng cần sống đủ ≥7 ngày mới qua.</t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="inlineStr">
-        <is>
-          <t>chưa có mốc bắt đầu</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="27" t="inlineStr">
-        <is>
-          <t>Chú giải: ✅ Đã qua ngưỡng · 🔶 Đang chạy · ⬜ Chưa bắt đầu. "Số ngày" của giai đoạn đang chạy tính tới hôm nay, tăng dần mỗi ngày cho tới khi chuyển giai đoạn kế tiếp.</t>
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Chú giải: cập nhật LAN_SUA_LON_CUOI trong script mỗi khi có commit đổi mã/CSDL thật — chuỗi yên tự reset về 0. "Sửa lớn" không tính commit chỉ đổi Timeline_Viet_Anh_Class.xlsx hoặc docs/*.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A9:D9"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D9">
+  <conditionalFormatting sqref="D6:D7">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>

</xml_diff>